<commit_message>
SEGUNDA SUBIDA DE PRUEBAS UNITARIAS Y/O CÓDIGOS by ELKIN
</commit_message>
<xml_diff>
--- a/CONEXIONES/conection.xlsx
+++ b/CONEXIONES/conection.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UNIVERSIDAD MECATRONICA\10 SEMESTRE MECATRONICA\CONTROL_INTELIGENTE_2\corte_1\conection\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNIVERSIDAD\2026-2\INTELIGENTE_II\Proyecto-Balanc-n-Inteligente-II\CONEXIONES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F2E0A974-9202-4828-B714-AC81D7323E79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{F1FD2A83-DF26-4FD2-BE4C-84BFE3000307}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -226,9 +225,6 @@
     <t>QTR-8A</t>
   </si>
   <si>
-    <t>OUT0</t>
-  </si>
-  <si>
     <t>GPIO1</t>
   </si>
   <si>
@@ -278,9 +274,6 @@
   </si>
   <si>
     <t>Así las salidas no superan el nivel del ESP32</t>
-  </si>
-  <si>
-    <t>LEDON</t>
   </si>
   <si>
     <t>Sin GPIO</t>
@@ -355,12 +348,18 @@
   <si>
     <t>GPIO48 mediante resistencia</t>
   </si>
+  <si>
+    <t>OUT8</t>
+  </si>
+  <si>
+    <t>LED_ON (IR)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -485,95 +484,95 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -590,6 +589,162 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>556161</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>38303</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>520777</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>22650</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9620992" y="3610797"/>
+          <a:ext cx="5506434" cy="5545957"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>778508</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>277790</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>79169</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagen 2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:srcRect r="66447"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10635027" y="0"/>
+          <a:ext cx="1874347" cy="3295403"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>381130</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>31120</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>170099</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>118993</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12612714" y="387380"/>
+          <a:ext cx="3747411" cy="2057197"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>149234</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>715530</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>154907</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Imagen 4"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8422377" y="0"/>
+          <a:ext cx="2149672" cy="3193011"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -888,17 +1043,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDFE5BFE-C806-443F-A859-297ADEE273FB}">
-  <dimension ref="A1:D47"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E47"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33" customWidth="1"/>
-    <col min="2" max="2" width="29.7109375" customWidth="1"/>
-    <col min="3" max="3" width="31.42578125" customWidth="1"/>
-    <col min="4" max="4" width="26.42578125" customWidth="1"/>
+    <col min="2" max="2" width="29.6640625" customWidth="1"/>
+    <col min="3" max="3" width="31.44140625" customWidth="1"/>
+    <col min="4" max="4" width="26.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -912,576 +1067,600 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="24"/>
+      <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="24"/>
+      <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="24"/>
+      <c r="B5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="3"/>
-      <c r="B6" s="4" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="24"/>
+      <c r="B6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="24"/>
+      <c r="B7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="30">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4" t="s">
+    <row r="8" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="24"/>
+      <c r="B8" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="24"/>
+      <c r="B9" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="3"/>
-      <c r="B10" s="4" t="s">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="24"/>
+      <c r="B10" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4" t="s">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="24"/>
+      <c r="B11" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="6" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="6"/>
-      <c r="B13" s="7" t="s">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="25"/>
+      <c r="B13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="6"/>
-      <c r="B14" s="7" t="s">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="25"/>
+      <c r="B14" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
-      <c r="A15" s="6"/>
-      <c r="B15" s="7" t="s">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="25"/>
+      <c r="B15" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="6"/>
-      <c r="B16" s="7" t="s">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="25"/>
+      <c r="B16" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="5" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="9" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="7" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
-      <c r="A18" s="9"/>
-      <c r="B18" s="10" t="s">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="23"/>
+      <c r="B18" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="7" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="9"/>
-      <c r="B19" s="10" t="s">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="23"/>
+      <c r="B19" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="7" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
-      <c r="A20" s="9"/>
-      <c r="B20" s="10" t="s">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="23"/>
+      <c r="B20" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
-      <c r="A21" s="9"/>
-      <c r="B21" s="10" t="s">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="23"/>
+      <c r="B21" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="7" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
-      <c r="A22" s="12" t="s">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C22" s="14" t="s">
+      <c r="C22" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="D22" s="13" t="s">
+      <c r="D22" s="9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
-      <c r="A23" s="12"/>
-      <c r="B23" s="13" t="s">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="26"/>
+      <c r="B23" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="C23" s="14" t="s">
+      <c r="C23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="D23" s="13" t="s">
+      <c r="D23" s="9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
-      <c r="A24" s="12"/>
-      <c r="B24" s="13" t="s">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="26"/>
+      <c r="B24" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C24" s="14" t="s">
+      <c r="C24" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="D24" s="13" t="s">
+      <c r="D24" s="9" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
-      <c r="A25" s="12"/>
-      <c r="B25" s="13" t="s">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="26"/>
+      <c r="B25" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C25" s="14" t="s">
+      <c r="C25" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D25" s="13" t="s">
+      <c r="D25" s="9" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
-      <c r="A26" s="12"/>
-      <c r="B26" s="13" t="s">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="26"/>
+      <c r="B26" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="C26" s="14" t="s">
+      <c r="C26" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="D26" s="9" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
-      <c r="A27" s="15" t="s">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="16" t="s">
+      <c r="B27" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C27" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="C27" s="17" t="s">
+      <c r="D27" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="D27" s="16" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4">
-      <c r="A28" s="15"/>
-      <c r="B28" s="16" t="s">
+      <c r="E27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="27"/>
+      <c r="B28" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C28" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="C28" s="17" t="s">
-        <v>63</v>
-      </c>
-      <c r="D28" s="16" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4">
-      <c r="A29" s="15"/>
-      <c r="B29" s="16" t="s">
+      <c r="D28" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="E28">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="27"/>
+      <c r="B29" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C29" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="C29" s="17" t="s">
-        <v>65</v>
-      </c>
-      <c r="D29" s="16" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4">
-      <c r="A30" s="15"/>
-      <c r="B30" s="16" t="s">
+      <c r="D29" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="E29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" s="27"/>
+      <c r="B30" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="C30" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="C30" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="D30" s="16" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="A31" s="15"/>
-      <c r="B31" s="16" t="s">
+      <c r="D30" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="E30">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" s="27"/>
+      <c r="B31" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="C31" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="C31" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="D31" s="16" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4">
-      <c r="A32" s="15"/>
-      <c r="B32" s="16" t="s">
+      <c r="D31" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="E31">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" s="27"/>
+      <c r="B32" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C32" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C32" s="17" t="s">
-        <v>71</v>
-      </c>
-      <c r="D32" s="16" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4">
-      <c r="A33" s="15"/>
-      <c r="B33" s="16" t="s">
+      <c r="D32" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="E32">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" s="27"/>
+      <c r="B33" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C33" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C33" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="D33" s="16" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4">
-      <c r="A34" s="15"/>
-      <c r="B34" s="16" t="s">
+      <c r="D33" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="E33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" s="27"/>
+      <c r="B34" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="C34" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="C34" s="17" t="s">
+      <c r="D34" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="E34">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A35" s="27"/>
+      <c r="B35" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D35" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="D34" s="16" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="30">
-      <c r="A35" s="15"/>
-      <c r="B35" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="C35" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="D35" s="16" t="s">
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" s="27"/>
+      <c r="B36" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C36" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D36" s="11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A37" s="27"/>
+      <c r="B37" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="C37" s="12" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="36" spans="1:4">
-      <c r="A36" s="15"/>
-      <c r="B36" s="16" t="s">
+      <c r="D37" s="11" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="B38" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C38" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="D38" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A39" s="28"/>
+      <c r="B39" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C39" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="C36" s="17" t="s">
+      <c r="D39" s="13" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" s="29" t="s">
+        <v>84</v>
+      </c>
+      <c r="B40" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="D40" s="15" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A41" s="29"/>
+      <c r="B41" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="C41" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D36" s="16" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="30">
-      <c r="A37" s="15"/>
-      <c r="B37" s="16" t="s">
-        <v>77</v>
-      </c>
-      <c r="C37" s="17" t="s">
-        <v>78</v>
-      </c>
-      <c r="D37" s="16" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4">
-      <c r="A38" s="18" t="s">
-        <v>80</v>
-      </c>
-      <c r="B38" s="19" t="s">
-        <v>81</v>
-      </c>
-      <c r="C38" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="D38" s="19" t="s">
+      <c r="D41" s="15" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
-      <c r="A39" s="18"/>
-      <c r="B39" s="19" t="s">
-        <v>84</v>
-      </c>
-      <c r="C39" s="20" t="s">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="B42" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="C42" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="D42" s="17" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" s="30"/>
+      <c r="B43" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="C43" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D39" s="19" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4">
-      <c r="A40" s="21" t="s">
-        <v>86</v>
-      </c>
-      <c r="B40" s="22" t="s">
-        <v>81</v>
-      </c>
-      <c r="C40" s="23" t="s">
-        <v>87</v>
-      </c>
-      <c r="D40" s="22" t="s">
+      <c r="D43" s="17" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="B44" s="19" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="41" spans="1:4">
-      <c r="A41" s="21"/>
-      <c r="B41" s="22" t="s">
-        <v>84</v>
-      </c>
-      <c r="C41" s="23" t="s">
+      <c r="C44" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="D44" s="19" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" s="31"/>
+      <c r="B45" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="C45" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="D41" s="22" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4">
-      <c r="A42" s="24" t="s">
-        <v>89</v>
-      </c>
-      <c r="B42" s="25" t="s">
+      <c r="D45" s="19" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="B46" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="C46" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="D46" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="C42" s="26" t="s">
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" s="32"/>
+      <c r="B47" s="21" t="s">
         <v>91</v>
       </c>
-      <c r="D42" s="25" t="s">
+      <c r="C47" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="D47" s="21" t="s">
         <v>92</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4">
-      <c r="A43" s="24"/>
-      <c r="B43" s="25" t="s">
-        <v>93</v>
-      </c>
-      <c r="C43" s="26" t="s">
-        <v>25</v>
-      </c>
-      <c r="D43" s="25" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4">
-      <c r="A44" s="27" t="s">
-        <v>95</v>
-      </c>
-      <c r="B44" s="28" t="s">
-        <v>90</v>
-      </c>
-      <c r="C44" s="29" t="s">
-        <v>96</v>
-      </c>
-      <c r="D44" s="28" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4">
-      <c r="A45" s="27"/>
-      <c r="B45" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="C45" s="29" t="s">
-        <v>25</v>
-      </c>
-      <c r="D45" s="28" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4">
-      <c r="A46" s="30" t="s">
-        <v>97</v>
-      </c>
-      <c r="B46" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="C46" s="32" t="s">
-        <v>98</v>
-      </c>
-      <c r="D46" s="31" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4">
-      <c r="A47" s="30"/>
-      <c r="B47" s="31" t="s">
-        <v>93</v>
-      </c>
-      <c r="C47" s="32" t="s">
-        <v>25</v>
-      </c>
-      <c r="D47" s="31" t="s">
-        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1498,5 +1677,6 @@
     <mergeCell ref="A27:A37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>